<commit_message>
Gap report: split into menu recipes vs sub-recipes, flag composites that already exist
Report now breaks recipes-with-gaps into 'Menu Recipes' vs 'Sub-Recipes (preps)' (preps = 0 gaps — all priced), adds each recipe's current cost, and flags composites that ALREADY exist as a recipe (link them) vs need creating. 5-sheet workbook + 5 CSVs + summary.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/CostCraft_Missing_Price_Report.xlsx
+++ b/reports/CostCraft_Missing_Price_Report.xlsx
@@ -3,10 +3,11 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Need Price" sheetId="1" r:id="rId1"/>
-    <sheet name="Make Sub-Recipe" sheetId="2" r:id="rId2"/>
-    <sheet name="Recipes With Gaps" sheetId="3" r:id="rId3"/>
-    <sheet name="Yields Missing Price" sheetId="4" r:id="rId4"/>
+    <sheet name="Menu Recipes With Gaps" sheetId="1" r:id="rId1"/>
+    <sheet name="Sub-Recipes With Gaps" sheetId="2" r:id="rId2"/>
+    <sheet name="Need Price (raw)" sheetId="3" r:id="rId3"/>
+    <sheet name="Make Sub-Recipe" sheetId="4" r:id="rId4"/>
+    <sheet name="Yields Missing Price" sheetId="5" r:id="rId5"/>
   </sheets>
 </workbook>
 </file>
@@ -400,6 +401,1238 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F60"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Recipe</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Brand</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Category</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Current Cost ₹</v>
+      </c>
+      <c r="E1" t="str">
+        <v># Missing</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Missing Ingredients</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Custom Stir Fry</v>
+      </c>
+      <c r="B2" t="str">
+        <v>aiko</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Mains</v>
+      </c>
+      <c r="D2">
+        <v>404.28</v>
+      </c>
+      <c r="E2">
+        <v>13</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Chilli Garlic Sauce - Wok hei sauce; Teriyaki Sauce - Sesame seed; Teriyaki Sauce - Water; Wok Hei Sauce - Black pepper; Wok Hei Sauce - Water; Yaki Soba Sauce - Black pepper; Yaki Soba Sauce - Corn starch; Yaki Soba Sauce - Crushed black pepper; Yaki Soba Sauce - Hot sauce; Yaki Soba Sauce - Oyster sauce; Yaki Soba Sauce - Soy sauce; Yaki Soba Sauce - Sugar; Yaki Soba Sauce - Water</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>New Dimsum Platter</v>
+      </c>
+      <c r="B3" t="str">
+        <v>aiko</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Dimsum</v>
+      </c>
+      <c r="D3">
+        <v>200.19</v>
+      </c>
+      <c r="E3">
+        <v>10</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Broad Beans; Cheese &amp; Chilli Dumplings; Chestnut Gyoza; Chili Crisp; Forest Dip; Forest Dumplings; Gyoza dip; Red Momos Sauce; Saucy Momos; Truffle Edamame Dumplings</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Gimbap 1</v>
+      </c>
+      <c r="B4" t="str">
+        <v>aiko</v>
+      </c>
+      <c r="C4" t="str">
+        <v>Sushi</v>
+      </c>
+      <c r="D4">
+        <v>111.12</v>
+      </c>
+      <c r="E4">
+        <v>5</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Fried Tofu toss on soy; Nori sheets; Pickled radish; Sautéed spinach with soy &amp; garlic; Unagi</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Shoyu Ramen</v>
+      </c>
+      <c r="B5" t="str">
+        <v>aiko</v>
+      </c>
+      <c r="C5" t="str">
+        <v>Noodles</v>
+      </c>
+      <c r="D5">
+        <v>42.6</v>
+      </c>
+      <c r="E5">
+        <v>5</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Dashi; Maida noodles; Scallion oil; Shoyu tare; Veg stock</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Cheese Chilli Dumplings</v>
+      </c>
+      <c r="B6" t="str">
+        <v>aiko</v>
+      </c>
+      <c r="C6" t="str">
+        <v>Dimsum</v>
+      </c>
+      <c r="D6">
+        <v>106.28</v>
+      </c>
+      <c r="E6">
+        <v>4</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Chestnut; Cumin powder; Hing; Pickled red Bhavnagri</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Chilli Oil Dumplings</v>
+      </c>
+      <c r="B7" t="str">
+        <v>aiko</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Dimsum</v>
+      </c>
+      <c r="D7">
+        <v>62.35</v>
+      </c>
+      <c r="E7">
+        <v>4</v>
+      </c>
+      <c r="F7" t="str">
+        <v>Chilli Oil Dumplings filling; Chilli Oil Dumplings paste; Fried glass noodles; Sichuan powder</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Kwispy Scallion Pancake</v>
+      </c>
+      <c r="B8" t="str">
+        <v>aiko</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Sides</v>
+      </c>
+      <c r="D8">
+        <v>9.58</v>
+      </c>
+      <c r="E8">
+        <v>4</v>
+      </c>
+      <c r="F8" t="str">
+        <v>Green garlic cream cheese; Scallion Pancake; Scallion salad; Sichuan soy glaze</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Lasagna</v>
+      </c>
+      <c r="B9" t="str">
+        <v>capiche</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Pasta</v>
+      </c>
+      <c r="D9">
+        <v>143.63</v>
+      </c>
+      <c r="E9">
+        <v>4</v>
+      </c>
+      <c r="F9" t="str">
+        <v>Celery (diced); Lasagna sheets (oven-ready); Nutmeg; Soy chunks (textured)</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Pasta Fritti 2.0</v>
+      </c>
+      <c r="B10" t="str">
+        <v>capiche</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Pasta</v>
+      </c>
+      <c r="D10">
+        <v>151.69</v>
+      </c>
+      <c r="E10">
+        <v>4</v>
+      </c>
+      <c r="F10" t="str">
+        <v>Batter; Pasta sheet 22 g x 2; Ricotta filling 15 g each; Seasoning</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Pistachio Mousse Cake</v>
+      </c>
+      <c r="B11" t="str">
+        <v>capiche</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Desserts</v>
+      </c>
+      <c r="D11">
+        <v>139.58</v>
+      </c>
+      <c r="E11">
+        <v>4</v>
+      </c>
+      <c r="F11" t="str">
+        <v>Kunafa base; Pistachio mousse; Pistachio sponge; White chocolate décor</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Tofu Bao</v>
+      </c>
+      <c r="B12" t="str">
+        <v>aiko</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Dimsum</v>
+      </c>
+      <c r="D12">
+        <v>40.95</v>
+      </c>
+      <c r="E12">
+        <v>4</v>
+      </c>
+      <c r="F12" t="str">
+        <v>Bao; Bao sauce base; Coleslaw; Tofu batter</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Bombay Blues Roll</v>
+      </c>
+      <c r="B13" t="str">
+        <v>aiko</v>
+      </c>
+      <c r="C13" t="str">
+        <v>Sushi</v>
+      </c>
+      <c r="D13">
+        <v>82.37</v>
+      </c>
+      <c r="E13">
+        <v>3</v>
+      </c>
+      <c r="F13" t="str">
+        <v>Nori; Salsa; Tempura flex</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Chestnut Gyoza</v>
+      </c>
+      <c r="B14" t="str">
+        <v>aiko</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Dimsum</v>
+      </c>
+      <c r="D14">
+        <v>64.05</v>
+      </c>
+      <c r="E14">
+        <v>3</v>
+      </c>
+      <c r="F14" t="str">
+        <v>Chestnut; Oil + Water (for steaming); Slurry</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>Drunken Noodles</v>
+      </c>
+      <c r="B15" t="str">
+        <v>aiko</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Noodles</v>
+      </c>
+      <c r="D15">
+        <v>38.55</v>
+      </c>
+      <c r="E15">
+        <v>3</v>
+      </c>
+      <c r="F15" t="str">
+        <v>Drunken sauce; Flat noodles; Mixed mushroom</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>General Tso's Water Chestnuts</v>
+      </c>
+      <c r="B16" t="str">
+        <v>aiko</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Sides</v>
+      </c>
+      <c r="D16">
+        <v>81.22</v>
+      </c>
+      <c r="E16">
+        <v>3</v>
+      </c>
+      <c r="F16" t="str">
+        <v>Drunken sauce; Gyoza dip; Water chestnut flour</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>Hakka Noodles</v>
+      </c>
+      <c r="B17" t="str">
+        <v>aiko</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Noodles</v>
+      </c>
+      <c r="D17">
+        <v>36.96</v>
+      </c>
+      <c r="E17">
+        <v>3</v>
+      </c>
+      <c r="F17" t="str">
+        <v>Boiled hakka noodles; Ginger-garlic paste; Hakka sauce</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>Okonomiyaki Gyoza (6 Pcs)</v>
+      </c>
+      <c r="B18" t="str">
+        <v>aiko</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Dimsum</v>
+      </c>
+      <c r="D18">
+        <v>118.72</v>
+      </c>
+      <c r="E18">
+        <v>3</v>
+      </c>
+      <c r="F18" t="str">
+        <v>Boiled soy keema; Chilli besan paste; Stock pwd</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>Thai Curry</v>
+      </c>
+      <c r="B19" t="str">
+        <v>aiko</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Mains</v>
+      </c>
+      <c r="D19">
+        <v>131.54</v>
+      </c>
+      <c r="E19">
+        <v>3</v>
+      </c>
+      <c r="F19" t="str">
+        <v>Green paste; Scallion oil; Sesame mix</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>Thai Spring Roll</v>
+      </c>
+      <c r="B20" t="str">
+        <v>aiko</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Appetiser</v>
+      </c>
+      <c r="D20">
+        <v>16.5</v>
+      </c>
+      <c r="E20">
+        <v>3</v>
+      </c>
+      <c r="F20" t="str">
+        <v>Black Vinegar; Sichuan Sauce; Thai Spring Filling</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>Volcano 1</v>
+      </c>
+      <c r="B21" t="str">
+        <v>aiko</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Sushi</v>
+      </c>
+      <c r="D21">
+        <v>118.69</v>
+      </c>
+      <c r="E21">
+        <v>3</v>
+      </c>
+      <c r="F21" t="str">
+        <v>Chilly crisps and oil; Nori sheet; Wasabi paste</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>Arancini</v>
+      </c>
+      <c r="B22" t="str">
+        <v>capiche</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Appetiser</v>
+      </c>
+      <c r="D22">
+        <v>48.04</v>
+      </c>
+      <c r="E22">
+        <v>2</v>
+      </c>
+      <c r="F22" t="str">
+        <v>Arancini batter; Cooked risotto rice mix</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>Caramelised Onion Pasta</v>
+      </c>
+      <c r="B23" t="str">
+        <v>capiche</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Pasta</v>
+      </c>
+      <c r="D23">
+        <v>62.24</v>
+      </c>
+      <c r="E23">
+        <v>2</v>
+      </c>
+      <c r="F23" t="str">
+        <v>1 ladle water; Mix seasoning</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>Creamy Corn Rocks</v>
+      </c>
+      <c r="B24" t="str">
+        <v>aiko</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Sides</v>
+      </c>
+      <c r="D24">
+        <v>71.65</v>
+      </c>
+      <c r="E24">
+        <v>2</v>
+      </c>
+      <c r="F24" t="str">
+        <v>Corn Rocks sauce; Sweet corn puree</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>Dragon Roll</v>
+      </c>
+      <c r="B25" t="str">
+        <v>aiko</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Sushi</v>
+      </c>
+      <c r="D25">
+        <v>86.42</v>
+      </c>
+      <c r="E25">
+        <v>2</v>
+      </c>
+      <c r="F25" t="str">
+        <v>Dragon sauce; Nori half sheet</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>Jalapeño Popper Roll</v>
+      </c>
+      <c r="B26" t="str">
+        <v>aiko</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Sushi</v>
+      </c>
+      <c r="D26">
+        <v>83.35</v>
+      </c>
+      <c r="E26">
+        <v>2</v>
+      </c>
+      <c r="F26" t="str">
+        <v>Fried spring roll; Nori</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>Korean Mandu</v>
+      </c>
+      <c r="B27" t="str">
+        <v>aiko</v>
+      </c>
+      <c r="C27" t="str">
+        <v>Sides</v>
+      </c>
+      <c r="D27">
+        <v>52.77</v>
+      </c>
+      <c r="E27">
+        <v>2</v>
+      </c>
+      <c r="F27" t="str">
+        <v>Julienne cut nori sheet; Korean Mandu filling</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>Kwispy Wonton</v>
+      </c>
+      <c r="B28" t="str">
+        <v>aiko</v>
+      </c>
+      <c r="C28" t="str">
+        <v>Appetiser</v>
+      </c>
+      <c r="D28">
+        <v>33.04</v>
+      </c>
+      <c r="E28">
+        <v>2</v>
+      </c>
+      <c r="F28" t="str">
+        <v>Chilli crisps; Kwispy Wonton filling</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>Pad Thai</v>
+      </c>
+      <c r="B29" t="str">
+        <v>aiko</v>
+      </c>
+      <c r="C29" t="str">
+        <v>Noodles</v>
+      </c>
+      <c r="D29">
+        <v>65.61</v>
+      </c>
+      <c r="E29">
+        <v>2</v>
+      </c>
+      <c r="F29" t="str">
+        <v>Ginger-garlic paste; Pad Thai sauce</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>Peanut Butter Ramen</v>
+      </c>
+      <c r="B30" t="str">
+        <v>aiko</v>
+      </c>
+      <c r="C30" t="str">
+        <v>Noodles</v>
+      </c>
+      <c r="D30">
+        <v>61.81</v>
+      </c>
+      <c r="E30">
+        <v>2</v>
+      </c>
+      <c r="F30" t="str">
+        <v>Ginger paste; Ramen noodles</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>Risotto</v>
+      </c>
+      <c r="B31" t="str">
+        <v>capiche</v>
+      </c>
+      <c r="C31" t="str">
+        <v>Pasta</v>
+      </c>
+      <c r="D31">
+        <v>134.96</v>
+      </c>
+      <c r="E31">
+        <v>2</v>
+      </c>
+      <c r="F31" t="str">
+        <v>Béchamel; Peas</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>Roasted Red Bell Pepper Soup</v>
+      </c>
+      <c r="B32" t="str">
+        <v>capiche</v>
+      </c>
+      <c r="C32" t="str">
+        <v>Soups</v>
+      </c>
+      <c r="D32">
+        <v>140.95</v>
+      </c>
+      <c r="E32">
+        <v>2</v>
+      </c>
+      <c r="F32" t="str">
+        <v>Roasted bell pepper paste; Sourdough</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>Saucy Brussels Sprouts</v>
+      </c>
+      <c r="B33" t="str">
+        <v>capiche</v>
+      </c>
+      <c r="C33" t="str">
+        <v>Vegetable</v>
+      </c>
+      <c r="D33">
+        <v>165.74</v>
+      </c>
+      <c r="E33">
+        <v>2</v>
+      </c>
+      <c r="F33" t="str">
+        <v>Plain mayonnaise; Salt &amp; black pepper</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>Spiced Miso Ramen</v>
+      </c>
+      <c r="B34" t="str">
+        <v>aiko</v>
+      </c>
+      <c r="C34" t="str">
+        <v>Noodles</v>
+      </c>
+      <c r="D34">
+        <v>84.77</v>
+      </c>
+      <c r="E34">
+        <v>2</v>
+      </c>
+      <c r="F34" t="str">
+        <v>Ginger paste; Ramen noodles</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>Sticky Toffee Pudding</v>
+      </c>
+      <c r="B35" t="str">
+        <v>capiche</v>
+      </c>
+      <c r="C35" t="str">
+        <v>Desserts</v>
+      </c>
+      <c r="D35">
+        <v>52.6</v>
+      </c>
+      <c r="E35">
+        <v>2</v>
+      </c>
+      <c r="F35" t="str">
+        <v>Caramel sauce; Sticky toffee pudding</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>Stuffed Conchiglioni</v>
+      </c>
+      <c r="B36" t="str">
+        <v>capiche</v>
+      </c>
+      <c r="C36" t="str">
+        <v>Pasta</v>
+      </c>
+      <c r="D36">
+        <v>103.03</v>
+      </c>
+      <c r="E36">
+        <v>2</v>
+      </c>
+      <c r="F36" t="str">
+        <v>Conchiglioni; Garlic pomodoro sauce</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>Tiramisu 3.0</v>
+      </c>
+      <c r="B37" t="str">
+        <v>capiche</v>
+      </c>
+      <c r="C37" t="str">
+        <v>Desserts</v>
+      </c>
+      <c r="D37">
+        <v>111.93</v>
+      </c>
+      <c r="E37">
+        <v>2</v>
+      </c>
+      <c r="F37" t="str">
+        <v>Coffee sponge; Tuile décor</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>Tokyo Style Pizza (Dough Base)</v>
+      </c>
+      <c r="B38" t="str">
+        <v>aiko</v>
+      </c>
+      <c r="C38" t="str">
+        <v>Pizza</v>
+      </c>
+      <c r="D38">
+        <v>536.3</v>
+      </c>
+      <c r="E38">
+        <v>2</v>
+      </c>
+      <c r="F38" t="str">
+        <v>Cold water; Water (Biga)</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>Alfredo Fettuccine</v>
+      </c>
+      <c r="B39" t="str">
+        <v>capiche</v>
+      </c>
+      <c r="C39" t="str">
+        <v>Pasta</v>
+      </c>
+      <c r="D39">
+        <v>71.69</v>
+      </c>
+      <c r="E39">
+        <v>1</v>
+      </c>
+      <c r="F39" t="str">
+        <v>Béchamel</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>Avocado Roll</v>
+      </c>
+      <c r="B40" t="str">
+        <v>aiko</v>
+      </c>
+      <c r="C40" t="str">
+        <v>Sushi</v>
+      </c>
+      <c r="D40">
+        <v>186.3</v>
+      </c>
+      <c r="E40">
+        <v>1</v>
+      </c>
+      <c r="F40" t="str">
+        <v>Nori</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>Brownie With Ice Cream</v>
+      </c>
+      <c r="B41" t="str">
+        <v>capiche</v>
+      </c>
+      <c r="C41" t="str">
+        <v>Desserts</v>
+      </c>
+      <c r="D41">
+        <v>108.15</v>
+      </c>
+      <c r="E41">
+        <v>1</v>
+      </c>
+      <c r="F41" t="str">
+        <v>Cookies &amp; cream ice cream</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>Buttery Chilli Garlic Noodles</v>
+      </c>
+      <c r="B42" t="str">
+        <v>aiko</v>
+      </c>
+      <c r="C42" t="str">
+        <v>Noodles</v>
+      </c>
+      <c r="D42">
+        <v>24.29</v>
+      </c>
+      <c r="E42">
+        <v>1</v>
+      </c>
+      <c r="F42" t="str">
+        <v>Boiled noodles</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>Caesar Salad</v>
+      </c>
+      <c r="B43" t="str">
+        <v>capiche</v>
+      </c>
+      <c r="C43" t="str">
+        <v>Salads</v>
+      </c>
+      <c r="D43">
+        <v>41.12</v>
+      </c>
+      <c r="E43">
+        <v>1</v>
+      </c>
+      <c r="F43" t="str">
+        <v>Caesar mayo</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>Cold Spicy Sesame Noodles</v>
+      </c>
+      <c r="B44" t="str">
+        <v>aiko</v>
+      </c>
+      <c r="C44" t="str">
+        <v>Noodles</v>
+      </c>
+      <c r="D44">
+        <v>71.18</v>
+      </c>
+      <c r="E44">
+        <v>1</v>
+      </c>
+      <c r="F44" t="str">
+        <v>Cold Spicy Sesame sauce</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>Corn Tempura Roll</v>
+      </c>
+      <c r="B45" t="str">
+        <v>aiko</v>
+      </c>
+      <c r="C45" t="str">
+        <v>Sushi</v>
+      </c>
+      <c r="D45">
+        <v>140.24</v>
+      </c>
+      <c r="E45">
+        <v>1</v>
+      </c>
+      <c r="F45" t="str">
+        <v>Nori</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>Garlic Bread</v>
+      </c>
+      <c r="B46" t="str">
+        <v>capiche</v>
+      </c>
+      <c r="C46" t="str">
+        <v>Appetiser</v>
+      </c>
+      <c r="D46">
+        <v>51.42</v>
+      </c>
+      <c r="E46">
+        <v>1</v>
+      </c>
+      <c r="F46" t="str">
+        <v>Bread base</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>Katsu Curry</v>
+      </c>
+      <c r="B47" t="str">
+        <v>aiko</v>
+      </c>
+      <c r="C47" t="str">
+        <v>Mains</v>
+      </c>
+      <c r="D47">
+        <v>36.46</v>
+      </c>
+      <c r="E47">
+        <v>1</v>
+      </c>
+      <c r="F47" t="str">
+        <v>Scallion oil</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>Kwispy Lotus Root</v>
+      </c>
+      <c r="B48" t="str">
+        <v>aiko</v>
+      </c>
+      <c r="C48" t="str">
+        <v>Sides</v>
+      </c>
+      <c r="D48">
+        <v>32.05</v>
+      </c>
+      <c r="E48">
+        <v>1</v>
+      </c>
+      <c r="F48" t="str">
+        <v>Lotus root sauce</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>Lemon Iced Tea</v>
+      </c>
+      <c r="B49" t="str">
+        <v>capiche</v>
+      </c>
+      <c r="C49" t="str">
+        <v>Drinks</v>
+      </c>
+      <c r="D49">
+        <v>14.66</v>
+      </c>
+      <c r="E49">
+        <v>1</v>
+      </c>
+      <c r="F49" t="str">
+        <v>Iced tea (Tata Gold)</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>Lemon Linguini</v>
+      </c>
+      <c r="B50" t="str">
+        <v>capiche</v>
+      </c>
+      <c r="C50" t="str">
+        <v>Pasta</v>
+      </c>
+      <c r="D50">
+        <v>115.65</v>
+      </c>
+      <c r="E50">
+        <v>1</v>
+      </c>
+      <c r="F50" t="str">
+        <v>Boiled linguini</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>Mint Mojito</v>
+      </c>
+      <c r="B51" t="str">
+        <v>capiche</v>
+      </c>
+      <c r="C51" t="str">
+        <v>Drinks</v>
+      </c>
+      <c r="D51">
+        <v>19.13</v>
+      </c>
+      <c r="E51">
+        <v>1</v>
+      </c>
+      <c r="F51" t="str">
+        <v>Kinley Soda</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>Miso Tomato Soup</v>
+      </c>
+      <c r="B52" t="str">
+        <v>capiche</v>
+      </c>
+      <c r="C52" t="str">
+        <v>Soups</v>
+      </c>
+      <c r="D52">
+        <v>47.14</v>
+      </c>
+      <c r="E52">
+        <v>1</v>
+      </c>
+      <c r="F52" t="str">
+        <v>Bay leaf (remove before blending)</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>Moscow Mule</v>
+      </c>
+      <c r="B53" t="str">
+        <v>capiche</v>
+      </c>
+      <c r="C53" t="str">
+        <v>Drinks</v>
+      </c>
+      <c r="D53">
+        <v>91.7</v>
+      </c>
+      <c r="E53">
+        <v>1</v>
+      </c>
+      <c r="F53" t="str">
+        <v>Gunsberg Ginger Beer</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>Pink Burrata Pasta</v>
+      </c>
+      <c r="B54" t="str">
+        <v>capiche</v>
+      </c>
+      <c r="C54" t="str">
+        <v>Pasta</v>
+      </c>
+      <c r="D54">
+        <v>124.8</v>
+      </c>
+      <c r="E54">
+        <v>1</v>
+      </c>
+      <c r="F54" t="str">
+        <v>Pumpkin seeds &amp; pistachios (crushed &amp; mixed)</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>Spicy Tomato &amp; Cream Macaroni</v>
+      </c>
+      <c r="B55" t="str">
+        <v>capiche</v>
+      </c>
+      <c r="C55" t="str">
+        <v>Pasta</v>
+      </c>
+      <c r="D55">
+        <v>71.94</v>
+      </c>
+      <c r="E55">
+        <v>1</v>
+      </c>
+      <c r="F55" t="str">
+        <v>Orange (creamy tomato) sauce</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>Steamed Edamame (Chilli / Salted)</v>
+      </c>
+      <c r="B56" t="str">
+        <v>aiko</v>
+      </c>
+      <c r="C56" t="str">
+        <v>Sides</v>
+      </c>
+      <c r="D56">
+        <v>104.77</v>
+      </c>
+      <c r="E56">
+        <v>1</v>
+      </c>
+      <c r="F56" t="str">
+        <v>Chilli Crisp (for chilli version)</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>Summer Burrata Salad</v>
+      </c>
+      <c r="B57" t="str">
+        <v>capiche</v>
+      </c>
+      <c r="C57" t="str">
+        <v>Salads</v>
+      </c>
+      <c r="D57">
+        <v>141.38</v>
+      </c>
+      <c r="E57">
+        <v>1</v>
+      </c>
+      <c r="F57" t="str">
+        <v>Granola (chopped)</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>Tamarind Fizz</v>
+      </c>
+      <c r="B58" t="str">
+        <v>capiche</v>
+      </c>
+      <c r="C58" t="str">
+        <v>Drinks</v>
+      </c>
+      <c r="D58">
+        <v>56.97</v>
+      </c>
+      <c r="E58">
+        <v>1</v>
+      </c>
+      <c r="F58" t="str">
+        <v>Tamarind syrup</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>Tomato Butter Risotto</v>
+      </c>
+      <c r="B59" t="str">
+        <v>capiche</v>
+      </c>
+      <c r="C59" t="str">
+        <v>Risotto</v>
+      </c>
+      <c r="D59">
+        <v>109.5</v>
+      </c>
+      <c r="E59">
+        <v>1</v>
+      </c>
+      <c r="F59" t="str">
+        <v>Pesto dollop</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>Tteokbokki</v>
+      </c>
+      <c r="B60" t="str">
+        <v>aiko</v>
+      </c>
+      <c r="C60" t="str">
+        <v>Sides</v>
+      </c>
+      <c r="D60">
+        <v>108.6</v>
+      </c>
+      <c r="E60">
+        <v>1</v>
+      </c>
+      <c r="F60" t="str">
+        <v>Tteokbokki sauce</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:F60"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:A2"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>(none)</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:A2"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E42"/>
   <sheetData>
     <row r="1">
@@ -1123,9 +2356,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D92"/>
+  <dimension ref="A1:E92"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1138,6 +2371,9 @@
         <v>Used in # Recipes</v>
       </c>
       <c r="D1" t="str">
+        <v>Already a recipe?</v>
+      </c>
+      <c r="E1" t="str">
         <v>Recipes</v>
       </c>
     </row>
@@ -1152,6 +2388,9 @@
         <v>3</v>
       </c>
       <c r="D2" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E2" t="str">
         <v>Katsu Curry; Shoyu Ramen; Thai Curry</v>
       </c>
     </row>
@@ -1166,6 +2405,9 @@
         <v>2</v>
       </c>
       <c r="D3" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E3" t="str">
         <v>Alfredo Fettuccine; Risotto</v>
       </c>
     </row>
@@ -1180,6 +2422,9 @@
         <v>2</v>
       </c>
       <c r="D4" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E4" t="str">
         <v>Drunken Noodles; General Tso's Water Chestnuts</v>
       </c>
     </row>
@@ -1194,6 +2439,9 @@
         <v>2</v>
       </c>
       <c r="D5" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E5" t="str">
         <v>Peanut Butter Ramen; Spiced Miso Ramen</v>
       </c>
     </row>
@@ -1208,6 +2456,9 @@
         <v>2</v>
       </c>
       <c r="D6" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E6" t="str">
         <v>Hakka Noodles; Pad Thai</v>
       </c>
     </row>
@@ -1222,6 +2473,9 @@
         <v>2</v>
       </c>
       <c r="D7" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E7" t="str">
         <v>General Tso's Water Chestnuts; New Dimsum Platter</v>
       </c>
     </row>
@@ -1236,6 +2490,9 @@
         <v>1</v>
       </c>
       <c r="D8" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E8" t="str">
         <v>Arancini</v>
       </c>
     </row>
@@ -1250,6 +2507,9 @@
         <v>1</v>
       </c>
       <c r="D9" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E9" t="str">
         <v>Tofu Bao</v>
       </c>
     </row>
@@ -1264,6 +2524,9 @@
         <v>1</v>
       </c>
       <c r="D10" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E10" t="str">
         <v>Pasta Fritti 2.0</v>
       </c>
     </row>
@@ -1278,6 +2541,9 @@
         <v>1</v>
       </c>
       <c r="D11" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E11" t="str">
         <v>Hakka Noodles</v>
       </c>
     </row>
@@ -1292,6 +2558,9 @@
         <v>1</v>
       </c>
       <c r="D12" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E12" t="str">
         <v>Buttery Chilli Garlic Noodles</v>
       </c>
     </row>
@@ -1306,6 +2575,9 @@
         <v>1</v>
       </c>
       <c r="D13" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E13" t="str">
         <v>Okonomiyaki Gyoza (6 Pcs)</v>
       </c>
     </row>
@@ -1320,6 +2592,9 @@
         <v>1</v>
       </c>
       <c r="D14" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E14" t="str">
         <v>Garlic Bread</v>
       </c>
     </row>
@@ -1334,6 +2609,9 @@
         <v>1</v>
       </c>
       <c r="D15" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E15" t="str">
         <v>Caesar Salad</v>
       </c>
     </row>
@@ -1348,6 +2626,9 @@
         <v>1</v>
       </c>
       <c r="D16" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E16" t="str">
         <v>Sticky Toffee Pudding</v>
       </c>
     </row>
@@ -1362,6 +2643,9 @@
         <v>1</v>
       </c>
       <c r="D17" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E17" t="str">
         <v>New Dimsum Platter</v>
       </c>
     </row>
@@ -1376,6 +2660,9 @@
         <v>1</v>
       </c>
       <c r="D18" t="str">
+        <v>YES — just link it</v>
+      </c>
+      <c r="E18" t="str">
         <v>New Dimsum Platter</v>
       </c>
     </row>
@@ -1390,6 +2677,9 @@
         <v>1</v>
       </c>
       <c r="D19" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E19" t="str">
         <v>New Dimsum Platter</v>
       </c>
     </row>
@@ -1404,6 +2694,9 @@
         <v>1</v>
       </c>
       <c r="D20" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E20" t="str">
         <v>Okonomiyaki Gyoza (6 Pcs)</v>
       </c>
     </row>
@@ -1418,6 +2711,9 @@
         <v>1</v>
       </c>
       <c r="D21" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E21" t="str">
         <v>Kwispy Wonton</v>
       </c>
     </row>
@@ -1432,6 +2728,9 @@
         <v>1</v>
       </c>
       <c r="D22" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E22" t="str">
         <v>Custom Stir Fry</v>
       </c>
     </row>
@@ -1446,6 +2745,9 @@
         <v>1</v>
       </c>
       <c r="D23" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E23" t="str">
         <v>Chilli Oil Dumplings</v>
       </c>
     </row>
@@ -1460,6 +2762,9 @@
         <v>1</v>
       </c>
       <c r="D24" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E24" t="str">
         <v>Chilli Oil Dumplings</v>
       </c>
     </row>
@@ -1474,6 +2779,9 @@
         <v>1</v>
       </c>
       <c r="D25" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E25" t="str">
         <v>Volcano 1</v>
       </c>
     </row>
@@ -1488,6 +2796,9 @@
         <v>1</v>
       </c>
       <c r="D26" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E26" t="str">
         <v>Tiramisu 3.0</v>
       </c>
     </row>
@@ -1502,6 +2813,9 @@
         <v>1</v>
       </c>
       <c r="D27" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E27" t="str">
         <v>Cold Spicy Sesame Noodles</v>
       </c>
     </row>
@@ -1516,6 +2830,9 @@
         <v>1</v>
       </c>
       <c r="D28" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E28" t="str">
         <v>Tofu Bao</v>
       </c>
     </row>
@@ -1530,6 +2847,9 @@
         <v>1</v>
       </c>
       <c r="D29" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E29" t="str">
         <v>Arancini</v>
       </c>
     </row>
@@ -1544,6 +2864,9 @@
         <v>1</v>
       </c>
       <c r="D30" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E30" t="str">
         <v>Creamy Corn Rocks</v>
       </c>
     </row>
@@ -1558,6 +2881,9 @@
         <v>1</v>
       </c>
       <c r="D31" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E31" t="str">
         <v>Shoyu Ramen</v>
       </c>
     </row>
@@ -1572,6 +2898,9 @@
         <v>1</v>
       </c>
       <c r="D32" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E32" t="str">
         <v>Dragon Roll</v>
       </c>
     </row>
@@ -1586,6 +2915,9 @@
         <v>1</v>
       </c>
       <c r="D33" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E33" t="str">
         <v>New Dimsum Platter</v>
       </c>
     </row>
@@ -1600,6 +2932,9 @@
         <v>1</v>
       </c>
       <c r="D34" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E34" t="str">
         <v>New Dimsum Platter</v>
       </c>
     </row>
@@ -1614,6 +2949,9 @@
         <v>1</v>
       </c>
       <c r="D35" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E35" t="str">
         <v>Jalapeño Popper Roll</v>
       </c>
     </row>
@@ -1628,6 +2966,9 @@
         <v>1</v>
       </c>
       <c r="D36" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E36" t="str">
         <v>Gimbap 1</v>
       </c>
     </row>
@@ -1642,6 +2983,9 @@
         <v>1</v>
       </c>
       <c r="D37" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E37" t="str">
         <v>Stuffed Conchiglioni</v>
       </c>
     </row>
@@ -1656,6 +3000,9 @@
         <v>1</v>
       </c>
       <c r="D38" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E38" t="str">
         <v>Kwispy Scallion Pancake</v>
       </c>
     </row>
@@ -1670,6 +3017,9 @@
         <v>1</v>
       </c>
       <c r="D39" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E39" t="str">
         <v>Thai Curry</v>
       </c>
     </row>
@@ -1684,6 +3034,9 @@
         <v>1</v>
       </c>
       <c r="D40" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E40" t="str">
         <v>Hakka Noodles</v>
       </c>
     </row>
@@ -1698,6 +3051,9 @@
         <v>1</v>
       </c>
       <c r="D41" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E41" t="str">
         <v>Lemon Iced Tea</v>
       </c>
     </row>
@@ -1712,6 +3068,9 @@
         <v>1</v>
       </c>
       <c r="D42" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E42" t="str">
         <v>Korean Mandu</v>
       </c>
     </row>
@@ -1726,6 +3085,9 @@
         <v>1</v>
       </c>
       <c r="D43" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E43" t="str">
         <v>Pistachio Mousse Cake</v>
       </c>
     </row>
@@ -1740,6 +3102,9 @@
         <v>1</v>
       </c>
       <c r="D44" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E44" t="str">
         <v>Kwispy Wonton</v>
       </c>
     </row>
@@ -1754,6 +3119,9 @@
         <v>1</v>
       </c>
       <c r="D45" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E45" t="str">
         <v>Kwispy Lotus Root</v>
       </c>
     </row>
@@ -1768,6 +3136,9 @@
         <v>1</v>
       </c>
       <c r="D46" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E46" t="str">
         <v>Caramelised Onion Pasta</v>
       </c>
     </row>
@@ -1782,6 +3153,9 @@
         <v>1</v>
       </c>
       <c r="D47" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E47" t="str">
         <v>Chestnut Gyoza</v>
       </c>
     </row>
@@ -1796,6 +3170,9 @@
         <v>1</v>
       </c>
       <c r="D48" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E48" t="str">
         <v>Spicy Tomato &amp; Cream Macaroni</v>
       </c>
     </row>
@@ -1810,6 +3187,9 @@
         <v>1</v>
       </c>
       <c r="D49" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E49" t="str">
         <v>Pad Thai</v>
       </c>
     </row>
@@ -1824,6 +3204,9 @@
         <v>1</v>
       </c>
       <c r="D50" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E50" t="str">
         <v>Tomato Butter Risotto</v>
       </c>
     </row>
@@ -1838,6 +3221,9 @@
         <v>1</v>
       </c>
       <c r="D51" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E51" t="str">
         <v>Pistachio Mousse Cake</v>
       </c>
     </row>
@@ -1852,6 +3238,9 @@
         <v>1</v>
       </c>
       <c r="D52" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E52" t="str">
         <v>Pistachio Mousse Cake</v>
       </c>
     </row>
@@ -1866,6 +3255,9 @@
         <v>1</v>
       </c>
       <c r="D53" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E53" t="str">
         <v>Pink Burrata Pasta</v>
       </c>
     </row>
@@ -1880,6 +3272,9 @@
         <v>1</v>
       </c>
       <c r="D54" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E54" t="str">
         <v>New Dimsum Platter</v>
       </c>
     </row>
@@ -1894,6 +3289,9 @@
         <v>1</v>
       </c>
       <c r="D55" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E55" t="str">
         <v>Pasta Fritti 2.0</v>
       </c>
     </row>
@@ -1908,6 +3306,9 @@
         <v>1</v>
       </c>
       <c r="D56" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E56" t="str">
         <v>Roasted Red Bell Pepper Soup</v>
       </c>
     </row>
@@ -1922,6 +3323,9 @@
         <v>1</v>
       </c>
       <c r="D57" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E57" t="str">
         <v>Bombay Blues Roll</v>
       </c>
     </row>
@@ -1936,6 +3340,9 @@
         <v>1</v>
       </c>
       <c r="D58" t="str">
+        <v>YES — just link it</v>
+      </c>
+      <c r="E58" t="str">
         <v>New Dimsum Platter</v>
       </c>
     </row>
@@ -1950,6 +3357,9 @@
         <v>1</v>
       </c>
       <c r="D59" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E59" t="str">
         <v>Gimbap 1</v>
       </c>
     </row>
@@ -1964,6 +3374,9 @@
         <v>1</v>
       </c>
       <c r="D60" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E60" t="str">
         <v>Kwispy Scallion Pancake</v>
       </c>
     </row>
@@ -1978,6 +3391,9 @@
         <v>1</v>
       </c>
       <c r="D61" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E61" t="str">
         <v>Kwispy Scallion Pancake</v>
       </c>
     </row>
@@ -1992,6 +3408,9 @@
         <v>1</v>
       </c>
       <c r="D62" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E62" t="str">
         <v>Pasta Fritti 2.0</v>
       </c>
     </row>
@@ -2006,6 +3425,9 @@
         <v>1</v>
       </c>
       <c r="D63" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E63" t="str">
         <v>Thai Curry</v>
       </c>
     </row>
@@ -2020,6 +3442,9 @@
         <v>1</v>
       </c>
       <c r="D64" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E64" t="str">
         <v>Shoyu Ramen</v>
       </c>
     </row>
@@ -2034,6 +3459,9 @@
         <v>1</v>
       </c>
       <c r="D65" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E65" t="str">
         <v>Thai Spring Roll</v>
       </c>
     </row>
@@ -2048,6 +3476,9 @@
         <v>1</v>
       </c>
       <c r="D66" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E66" t="str">
         <v>Kwispy Scallion Pancake</v>
       </c>
     </row>
@@ -2062,6 +3493,9 @@
         <v>1</v>
       </c>
       <c r="D67" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E67" t="str">
         <v>Chestnut Gyoza</v>
       </c>
     </row>
@@ -2076,6 +3510,9 @@
         <v>1</v>
       </c>
       <c r="D68" t="str">
+        <v>YES — just link it</v>
+      </c>
+      <c r="E68" t="str">
         <v>Sticky Toffee Pudding</v>
       </c>
     </row>
@@ -2090,6 +3527,9 @@
         <v>1</v>
       </c>
       <c r="D69" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E69" t="str">
         <v>Okonomiyaki Gyoza (6 Pcs)</v>
       </c>
     </row>
@@ -2104,6 +3544,9 @@
         <v>1</v>
       </c>
       <c r="D70" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E70" t="str">
         <v>Creamy Corn Rocks</v>
       </c>
     </row>
@@ -2118,6 +3561,9 @@
         <v>1</v>
       </c>
       <c r="D71" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E71" t="str">
         <v>Tamarind Fizz</v>
       </c>
     </row>
@@ -2132,6 +3578,9 @@
         <v>1</v>
       </c>
       <c r="D72" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E72" t="str">
         <v>Bombay Blues Roll</v>
       </c>
     </row>
@@ -2146,6 +3595,9 @@
         <v>1</v>
       </c>
       <c r="D73" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E73" t="str">
         <v>Custom Stir Fry</v>
       </c>
     </row>
@@ -2160,6 +3612,9 @@
         <v>1</v>
       </c>
       <c r="D74" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E74" t="str">
         <v>Custom Stir Fry</v>
       </c>
     </row>
@@ -2174,6 +3629,9 @@
         <v>1</v>
       </c>
       <c r="D75" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E75" t="str">
         <v>Thai Spring Roll</v>
       </c>
     </row>
@@ -2188,6 +3646,9 @@
         <v>1</v>
       </c>
       <c r="D76" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E76" t="str">
         <v>Tofu Bao</v>
       </c>
     </row>
@@ -2202,6 +3663,9 @@
         <v>1</v>
       </c>
       <c r="D77" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E77" t="str">
         <v>New Dimsum Platter</v>
       </c>
     </row>
@@ -2216,6 +3680,9 @@
         <v>1</v>
       </c>
       <c r="D78" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E78" t="str">
         <v>Tteokbokki</v>
       </c>
     </row>
@@ -2230,6 +3697,9 @@
         <v>1</v>
       </c>
       <c r="D79" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E79" t="str">
         <v>Tiramisu 3.0</v>
       </c>
     </row>
@@ -2244,6 +3714,9 @@
         <v>1</v>
       </c>
       <c r="D80" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E80" t="str">
         <v>Shoyu Ramen</v>
       </c>
     </row>
@@ -2258,6 +3731,9 @@
         <v>1</v>
       </c>
       <c r="D81" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E81" t="str">
         <v>Volcano 1</v>
       </c>
     </row>
@@ -2272,6 +3748,9 @@
         <v>1</v>
       </c>
       <c r="D82" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E82" t="str">
         <v>Pistachio Mousse Cake</v>
       </c>
     </row>
@@ -2286,6 +3765,9 @@
         <v>1</v>
       </c>
       <c r="D83" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E83" t="str">
         <v>Custom Stir Fry</v>
       </c>
     </row>
@@ -2300,6 +3782,9 @@
         <v>1</v>
       </c>
       <c r="D84" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E84" t="str">
         <v>Custom Stir Fry</v>
       </c>
     </row>
@@ -2314,6 +3799,9 @@
         <v>1</v>
       </c>
       <c r="D85" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E85" t="str">
         <v>Custom Stir Fry</v>
       </c>
     </row>
@@ -2328,6 +3816,9 @@
         <v>1</v>
       </c>
       <c r="D86" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E86" t="str">
         <v>Custom Stir Fry</v>
       </c>
     </row>
@@ -2342,6 +3833,9 @@
         <v>1</v>
       </c>
       <c r="D87" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E87" t="str">
         <v>Custom Stir Fry</v>
       </c>
     </row>
@@ -2356,6 +3850,9 @@
         <v>1</v>
       </c>
       <c r="D88" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E88" t="str">
         <v>Custom Stir Fry</v>
       </c>
     </row>
@@ -2370,6 +3867,9 @@
         <v>1</v>
       </c>
       <c r="D89" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E89" t="str">
         <v>Custom Stir Fry</v>
       </c>
     </row>
@@ -2384,6 +3884,9 @@
         <v>1</v>
       </c>
       <c r="D90" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E90" t="str">
         <v>Custom Stir Fry</v>
       </c>
     </row>
@@ -2398,6 +3901,9 @@
         <v>1</v>
       </c>
       <c r="D91" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E91" t="str">
         <v>Custom Stir Fry</v>
       </c>
     </row>
@@ -2412,1048 +3918,20 @@
         <v>1</v>
       </c>
       <c r="D92" t="str">
+        <v>no — create it</v>
+      </c>
+      <c r="E92" t="str">
         <v>Custom Stir Fry</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D92"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E92"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E60"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Recipe</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Brand</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Category</v>
-      </c>
-      <c r="D1" t="str">
-        <v># Missing</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Missing Ingredients</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>Custom Stir Fry</v>
-      </c>
-      <c r="B2" t="str">
-        <v>aiko</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Mains</v>
-      </c>
-      <c r="D2">
-        <v>13</v>
-      </c>
-      <c r="E2" t="str">
-        <v>Chilli Garlic Sauce - Wok hei sauce; Teriyaki Sauce - Sesame seed; Teriyaki Sauce - Water; Wok Hei Sauce - Black pepper; Wok Hei Sauce - Water; Yaki Soba Sauce - Black pepper; Yaki Soba Sauce - Corn starch; Yaki Soba Sauce - Crushed black pepper; Yaki Soba Sauce - Hot sauce; Yaki Soba Sauce - Oyster sauce; Yaki Soba Sauce - Soy sauce; Yaki Soba Sauce - Sugar; Yaki Soba Sauce - Water</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>New Dimsum Platter</v>
-      </c>
-      <c r="B3" t="str">
-        <v>aiko</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Dimsum</v>
-      </c>
-      <c r="D3">
-        <v>10</v>
-      </c>
-      <c r="E3" t="str">
-        <v>Broad Beans; Cheese &amp; Chilli Dumplings; Chestnut Gyoza; Chili Crisp; Forest Dip; Forest Dumplings; Gyoza dip; Red Momos Sauce; Saucy Momos; Truffle Edamame Dumplings</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Gimbap 1</v>
-      </c>
-      <c r="B4" t="str">
-        <v>aiko</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Sushi</v>
-      </c>
-      <c r="D4">
-        <v>5</v>
-      </c>
-      <c r="E4" t="str">
-        <v>Fried Tofu toss on soy; Nori sheets; Pickled radish; Sautéed spinach with soy &amp; garlic; Unagi</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>Shoyu Ramen</v>
-      </c>
-      <c r="B5" t="str">
-        <v>aiko</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Noodles</v>
-      </c>
-      <c r="D5">
-        <v>5</v>
-      </c>
-      <c r="E5" t="str">
-        <v>Dashi; Maida noodles; Scallion oil; Shoyu tare; Veg stock</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>Cheese Chilli Dumplings</v>
-      </c>
-      <c r="B6" t="str">
-        <v>aiko</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Dimsum</v>
-      </c>
-      <c r="D6">
-        <v>4</v>
-      </c>
-      <c r="E6" t="str">
-        <v>Chestnut; Cumin powder; Hing; Pickled red Bhavnagri</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>Chilli Oil Dumplings</v>
-      </c>
-      <c r="B7" t="str">
-        <v>aiko</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Dimsum</v>
-      </c>
-      <c r="D7">
-        <v>4</v>
-      </c>
-      <c r="E7" t="str">
-        <v>Chilli Oil Dumplings filling; Chilli Oil Dumplings paste; Fried glass noodles; Sichuan powder</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>Kwispy Scallion Pancake</v>
-      </c>
-      <c r="B8" t="str">
-        <v>aiko</v>
-      </c>
-      <c r="C8" t="str">
-        <v>Sides</v>
-      </c>
-      <c r="D8">
-        <v>4</v>
-      </c>
-      <c r="E8" t="str">
-        <v>Green garlic cream cheese; Scallion Pancake; Scallion salad; Sichuan soy glaze</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>Lasagna</v>
-      </c>
-      <c r="B9" t="str">
-        <v>capiche</v>
-      </c>
-      <c r="C9" t="str">
-        <v>Pasta</v>
-      </c>
-      <c r="D9">
-        <v>4</v>
-      </c>
-      <c r="E9" t="str">
-        <v>Celery (diced); Lasagna sheets (oven-ready); Nutmeg; Soy chunks (textured)</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>Pasta Fritti 2.0</v>
-      </c>
-      <c r="B10" t="str">
-        <v>capiche</v>
-      </c>
-      <c r="C10" t="str">
-        <v>Pasta</v>
-      </c>
-      <c r="D10">
-        <v>4</v>
-      </c>
-      <c r="E10" t="str">
-        <v>Batter; Pasta sheet 22 g x 2; Ricotta filling 15 g each; Seasoning</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>Pistachio Mousse Cake</v>
-      </c>
-      <c r="B11" t="str">
-        <v>capiche</v>
-      </c>
-      <c r="C11" t="str">
-        <v>Desserts</v>
-      </c>
-      <c r="D11">
-        <v>4</v>
-      </c>
-      <c r="E11" t="str">
-        <v>Kunafa base; Pistachio mousse; Pistachio sponge; White chocolate décor</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>Tofu Bao</v>
-      </c>
-      <c r="B12" t="str">
-        <v>aiko</v>
-      </c>
-      <c r="C12" t="str">
-        <v>Dimsum</v>
-      </c>
-      <c r="D12">
-        <v>4</v>
-      </c>
-      <c r="E12" t="str">
-        <v>Bao; Bao sauce base; Coleslaw; Tofu batter</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>Bombay Blues Roll</v>
-      </c>
-      <c r="B13" t="str">
-        <v>aiko</v>
-      </c>
-      <c r="C13" t="str">
-        <v>Sushi</v>
-      </c>
-      <c r="D13">
-        <v>3</v>
-      </c>
-      <c r="E13" t="str">
-        <v>Nori; Salsa; Tempura flex</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v>Chestnut Gyoza</v>
-      </c>
-      <c r="B14" t="str">
-        <v>aiko</v>
-      </c>
-      <c r="C14" t="str">
-        <v>Dimsum</v>
-      </c>
-      <c r="D14">
-        <v>3</v>
-      </c>
-      <c r="E14" t="str">
-        <v>Chestnut; Oil + Water (for steaming); Slurry</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="str">
-        <v>Drunken Noodles</v>
-      </c>
-      <c r="B15" t="str">
-        <v>aiko</v>
-      </c>
-      <c r="C15" t="str">
-        <v>Noodles</v>
-      </c>
-      <c r="D15">
-        <v>3</v>
-      </c>
-      <c r="E15" t="str">
-        <v>Drunken sauce; Flat noodles; Mixed mushroom</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="str">
-        <v>General Tso's Water Chestnuts</v>
-      </c>
-      <c r="B16" t="str">
-        <v>aiko</v>
-      </c>
-      <c r="C16" t="str">
-        <v>Sides</v>
-      </c>
-      <c r="D16">
-        <v>3</v>
-      </c>
-      <c r="E16" t="str">
-        <v>Drunken sauce; Gyoza dip; Water chestnut flour</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="str">
-        <v>Hakka Noodles</v>
-      </c>
-      <c r="B17" t="str">
-        <v>aiko</v>
-      </c>
-      <c r="C17" t="str">
-        <v>Noodles</v>
-      </c>
-      <c r="D17">
-        <v>3</v>
-      </c>
-      <c r="E17" t="str">
-        <v>Boiled hakka noodles; Ginger-garlic paste; Hakka sauce</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="str">
-        <v>Okonomiyaki Gyoza (6 Pcs)</v>
-      </c>
-      <c r="B18" t="str">
-        <v>aiko</v>
-      </c>
-      <c r="C18" t="str">
-        <v>Dimsum</v>
-      </c>
-      <c r="D18">
-        <v>3</v>
-      </c>
-      <c r="E18" t="str">
-        <v>Boiled soy keema; Chilli besan paste; Stock pwd</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="str">
-        <v>Thai Curry</v>
-      </c>
-      <c r="B19" t="str">
-        <v>aiko</v>
-      </c>
-      <c r="C19" t="str">
-        <v>Mains</v>
-      </c>
-      <c r="D19">
-        <v>3</v>
-      </c>
-      <c r="E19" t="str">
-        <v>Green paste; Scallion oil; Sesame mix</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="str">
-        <v>Thai Spring Roll</v>
-      </c>
-      <c r="B20" t="str">
-        <v>aiko</v>
-      </c>
-      <c r="C20" t="str">
-        <v>Appetiser</v>
-      </c>
-      <c r="D20">
-        <v>3</v>
-      </c>
-      <c r="E20" t="str">
-        <v>Black Vinegar; Sichuan Sauce; Thai Spring Filling</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="str">
-        <v>Volcano 1</v>
-      </c>
-      <c r="B21" t="str">
-        <v>aiko</v>
-      </c>
-      <c r="C21" t="str">
-        <v>Sushi</v>
-      </c>
-      <c r="D21">
-        <v>3</v>
-      </c>
-      <c r="E21" t="str">
-        <v>Chilly crisps and oil; Nori sheet; Wasabi paste</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="str">
-        <v>Arancini</v>
-      </c>
-      <c r="B22" t="str">
-        <v>capiche</v>
-      </c>
-      <c r="C22" t="str">
-        <v>Appetiser</v>
-      </c>
-      <c r="D22">
-        <v>2</v>
-      </c>
-      <c r="E22" t="str">
-        <v>Arancini batter; Cooked risotto rice mix</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="str">
-        <v>Caramelised Onion Pasta</v>
-      </c>
-      <c r="B23" t="str">
-        <v>capiche</v>
-      </c>
-      <c r="C23" t="str">
-        <v>Pasta</v>
-      </c>
-      <c r="D23">
-        <v>2</v>
-      </c>
-      <c r="E23" t="str">
-        <v>1 ladle water; Mix seasoning</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="str">
-        <v>Creamy Corn Rocks</v>
-      </c>
-      <c r="B24" t="str">
-        <v>aiko</v>
-      </c>
-      <c r="C24" t="str">
-        <v>Sides</v>
-      </c>
-      <c r="D24">
-        <v>2</v>
-      </c>
-      <c r="E24" t="str">
-        <v>Corn Rocks sauce; Sweet corn puree</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="str">
-        <v>Dragon Roll</v>
-      </c>
-      <c r="B25" t="str">
-        <v>aiko</v>
-      </c>
-      <c r="C25" t="str">
-        <v>Sushi</v>
-      </c>
-      <c r="D25">
-        <v>2</v>
-      </c>
-      <c r="E25" t="str">
-        <v>Dragon sauce; Nori half sheet</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="str">
-        <v>Jalapeño Popper Roll</v>
-      </c>
-      <c r="B26" t="str">
-        <v>aiko</v>
-      </c>
-      <c r="C26" t="str">
-        <v>Sushi</v>
-      </c>
-      <c r="D26">
-        <v>2</v>
-      </c>
-      <c r="E26" t="str">
-        <v>Fried spring roll; Nori</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="str">
-        <v>Korean Mandu</v>
-      </c>
-      <c r="B27" t="str">
-        <v>aiko</v>
-      </c>
-      <c r="C27" t="str">
-        <v>Sides</v>
-      </c>
-      <c r="D27">
-        <v>2</v>
-      </c>
-      <c r="E27" t="str">
-        <v>Julienne cut nori sheet; Korean Mandu filling</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="str">
-        <v>Kwispy Wonton</v>
-      </c>
-      <c r="B28" t="str">
-        <v>aiko</v>
-      </c>
-      <c r="C28" t="str">
-        <v>Appetiser</v>
-      </c>
-      <c r="D28">
-        <v>2</v>
-      </c>
-      <c r="E28" t="str">
-        <v>Chilli crisps; Kwispy Wonton filling</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="str">
-        <v>Pad Thai</v>
-      </c>
-      <c r="B29" t="str">
-        <v>aiko</v>
-      </c>
-      <c r="C29" t="str">
-        <v>Noodles</v>
-      </c>
-      <c r="D29">
-        <v>2</v>
-      </c>
-      <c r="E29" t="str">
-        <v>Ginger-garlic paste; Pad Thai sauce</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="str">
-        <v>Peanut Butter Ramen</v>
-      </c>
-      <c r="B30" t="str">
-        <v>aiko</v>
-      </c>
-      <c r="C30" t="str">
-        <v>Noodles</v>
-      </c>
-      <c r="D30">
-        <v>2</v>
-      </c>
-      <c r="E30" t="str">
-        <v>Ginger paste; Ramen noodles</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="str">
-        <v>Risotto</v>
-      </c>
-      <c r="B31" t="str">
-        <v>capiche</v>
-      </c>
-      <c r="C31" t="str">
-        <v>Pasta</v>
-      </c>
-      <c r="D31">
-        <v>2</v>
-      </c>
-      <c r="E31" t="str">
-        <v>Béchamel; Peas</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="str">
-        <v>Roasted Red Bell Pepper Soup</v>
-      </c>
-      <c r="B32" t="str">
-        <v>capiche</v>
-      </c>
-      <c r="C32" t="str">
-        <v>Soups</v>
-      </c>
-      <c r="D32">
-        <v>2</v>
-      </c>
-      <c r="E32" t="str">
-        <v>Roasted bell pepper paste; Sourdough</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="str">
-        <v>Saucy Brussels Sprouts</v>
-      </c>
-      <c r="B33" t="str">
-        <v>capiche</v>
-      </c>
-      <c r="C33" t="str">
-        <v>Vegetable</v>
-      </c>
-      <c r="D33">
-        <v>2</v>
-      </c>
-      <c r="E33" t="str">
-        <v>Plain mayonnaise; Salt &amp; black pepper</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="str">
-        <v>Spiced Miso Ramen</v>
-      </c>
-      <c r="B34" t="str">
-        <v>aiko</v>
-      </c>
-      <c r="C34" t="str">
-        <v>Noodles</v>
-      </c>
-      <c r="D34">
-        <v>2</v>
-      </c>
-      <c r="E34" t="str">
-        <v>Ginger paste; Ramen noodles</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="str">
-        <v>Sticky Toffee Pudding</v>
-      </c>
-      <c r="B35" t="str">
-        <v>capiche</v>
-      </c>
-      <c r="C35" t="str">
-        <v>Desserts</v>
-      </c>
-      <c r="D35">
-        <v>2</v>
-      </c>
-      <c r="E35" t="str">
-        <v>Caramel sauce; Sticky toffee pudding</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="str">
-        <v>Stuffed Conchiglioni</v>
-      </c>
-      <c r="B36" t="str">
-        <v>capiche</v>
-      </c>
-      <c r="C36" t="str">
-        <v>Pasta</v>
-      </c>
-      <c r="D36">
-        <v>2</v>
-      </c>
-      <c r="E36" t="str">
-        <v>Conchiglioni; Garlic pomodoro sauce</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="str">
-        <v>Tiramisu 3.0</v>
-      </c>
-      <c r="B37" t="str">
-        <v>capiche</v>
-      </c>
-      <c r="C37" t="str">
-        <v>Desserts</v>
-      </c>
-      <c r="D37">
-        <v>2</v>
-      </c>
-      <c r="E37" t="str">
-        <v>Coffee sponge; Tuile décor</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="str">
-        <v>Tokyo Style Pizza (Dough Base)</v>
-      </c>
-      <c r="B38" t="str">
-        <v>aiko</v>
-      </c>
-      <c r="C38" t="str">
-        <v>Pizza</v>
-      </c>
-      <c r="D38">
-        <v>2</v>
-      </c>
-      <c r="E38" t="str">
-        <v>Cold water; Water (Biga)</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="str">
-        <v>Alfredo Fettuccine</v>
-      </c>
-      <c r="B39" t="str">
-        <v>capiche</v>
-      </c>
-      <c r="C39" t="str">
-        <v>Pasta</v>
-      </c>
-      <c r="D39">
-        <v>1</v>
-      </c>
-      <c r="E39" t="str">
-        <v>Béchamel</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="str">
-        <v>Avocado Roll</v>
-      </c>
-      <c r="B40" t="str">
-        <v>aiko</v>
-      </c>
-      <c r="C40" t="str">
-        <v>Sushi</v>
-      </c>
-      <c r="D40">
-        <v>1</v>
-      </c>
-      <c r="E40" t="str">
-        <v>Nori</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="str">
-        <v>Brownie With Ice Cream</v>
-      </c>
-      <c r="B41" t="str">
-        <v>capiche</v>
-      </c>
-      <c r="C41" t="str">
-        <v>Desserts</v>
-      </c>
-      <c r="D41">
-        <v>1</v>
-      </c>
-      <c r="E41" t="str">
-        <v>Cookies &amp; cream ice cream</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="str">
-        <v>Buttery Chilli Garlic Noodles</v>
-      </c>
-      <c r="B42" t="str">
-        <v>aiko</v>
-      </c>
-      <c r="C42" t="str">
-        <v>Noodles</v>
-      </c>
-      <c r="D42">
-        <v>1</v>
-      </c>
-      <c r="E42" t="str">
-        <v>Boiled noodles</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="str">
-        <v>Caesar Salad</v>
-      </c>
-      <c r="B43" t="str">
-        <v>capiche</v>
-      </c>
-      <c r="C43" t="str">
-        <v>Salads</v>
-      </c>
-      <c r="D43">
-        <v>1</v>
-      </c>
-      <c r="E43" t="str">
-        <v>Caesar mayo</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="str">
-        <v>Cold Spicy Sesame Noodles</v>
-      </c>
-      <c r="B44" t="str">
-        <v>aiko</v>
-      </c>
-      <c r="C44" t="str">
-        <v>Noodles</v>
-      </c>
-      <c r="D44">
-        <v>1</v>
-      </c>
-      <c r="E44" t="str">
-        <v>Cold Spicy Sesame sauce</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="str">
-        <v>Corn Tempura Roll</v>
-      </c>
-      <c r="B45" t="str">
-        <v>aiko</v>
-      </c>
-      <c r="C45" t="str">
-        <v>Sushi</v>
-      </c>
-      <c r="D45">
-        <v>1</v>
-      </c>
-      <c r="E45" t="str">
-        <v>Nori</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="str">
-        <v>Garlic Bread</v>
-      </c>
-      <c r="B46" t="str">
-        <v>capiche</v>
-      </c>
-      <c r="C46" t="str">
-        <v>Appetiser</v>
-      </c>
-      <c r="D46">
-        <v>1</v>
-      </c>
-      <c r="E46" t="str">
-        <v>Bread base</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="str">
-        <v>Katsu Curry</v>
-      </c>
-      <c r="B47" t="str">
-        <v>aiko</v>
-      </c>
-      <c r="C47" t="str">
-        <v>Mains</v>
-      </c>
-      <c r="D47">
-        <v>1</v>
-      </c>
-      <c r="E47" t="str">
-        <v>Scallion oil</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="str">
-        <v>Kwispy Lotus Root</v>
-      </c>
-      <c r="B48" t="str">
-        <v>aiko</v>
-      </c>
-      <c r="C48" t="str">
-        <v>Sides</v>
-      </c>
-      <c r="D48">
-        <v>1</v>
-      </c>
-      <c r="E48" t="str">
-        <v>Lotus root sauce</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="str">
-        <v>Lemon Iced Tea</v>
-      </c>
-      <c r="B49" t="str">
-        <v>capiche</v>
-      </c>
-      <c r="C49" t="str">
-        <v>Drinks</v>
-      </c>
-      <c r="D49">
-        <v>1</v>
-      </c>
-      <c r="E49" t="str">
-        <v>Iced tea (Tata Gold)</v>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="str">
-        <v>Lemon Linguini</v>
-      </c>
-      <c r="B50" t="str">
-        <v>capiche</v>
-      </c>
-      <c r="C50" t="str">
-        <v>Pasta</v>
-      </c>
-      <c r="D50">
-        <v>1</v>
-      </c>
-      <c r="E50" t="str">
-        <v>Boiled linguini</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="str">
-        <v>Mint Mojito</v>
-      </c>
-      <c r="B51" t="str">
-        <v>capiche</v>
-      </c>
-      <c r="C51" t="str">
-        <v>Drinks</v>
-      </c>
-      <c r="D51">
-        <v>1</v>
-      </c>
-      <c r="E51" t="str">
-        <v>Kinley Soda</v>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="str">
-        <v>Miso Tomato Soup</v>
-      </c>
-      <c r="B52" t="str">
-        <v>capiche</v>
-      </c>
-      <c r="C52" t="str">
-        <v>Soups</v>
-      </c>
-      <c r="D52">
-        <v>1</v>
-      </c>
-      <c r="E52" t="str">
-        <v>Bay leaf (remove before blending)</v>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="str">
-        <v>Moscow Mule</v>
-      </c>
-      <c r="B53" t="str">
-        <v>capiche</v>
-      </c>
-      <c r="C53" t="str">
-        <v>Drinks</v>
-      </c>
-      <c r="D53">
-        <v>1</v>
-      </c>
-      <c r="E53" t="str">
-        <v>Gunsberg Ginger Beer</v>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="str">
-        <v>Pink Burrata Pasta</v>
-      </c>
-      <c r="B54" t="str">
-        <v>capiche</v>
-      </c>
-      <c r="C54" t="str">
-        <v>Pasta</v>
-      </c>
-      <c r="D54">
-        <v>1</v>
-      </c>
-      <c r="E54" t="str">
-        <v>Pumpkin seeds &amp; pistachios (crushed &amp; mixed)</v>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="str">
-        <v>Spicy Tomato &amp; Cream Macaroni</v>
-      </c>
-      <c r="B55" t="str">
-        <v>capiche</v>
-      </c>
-      <c r="C55" t="str">
-        <v>Pasta</v>
-      </c>
-      <c r="D55">
-        <v>1</v>
-      </c>
-      <c r="E55" t="str">
-        <v>Orange (creamy tomato) sauce</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="str">
-        <v>Steamed Edamame (Chilli / Salted)</v>
-      </c>
-      <c r="B56" t="str">
-        <v>aiko</v>
-      </c>
-      <c r="C56" t="str">
-        <v>Sides</v>
-      </c>
-      <c r="D56">
-        <v>1</v>
-      </c>
-      <c r="E56" t="str">
-        <v>Chilli Crisp (for chilli version)</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="str">
-        <v>Summer Burrata Salad</v>
-      </c>
-      <c r="B57" t="str">
-        <v>capiche</v>
-      </c>
-      <c r="C57" t="str">
-        <v>Salads</v>
-      </c>
-      <c r="D57">
-        <v>1</v>
-      </c>
-      <c r="E57" t="str">
-        <v>Granola (chopped)</v>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="str">
-        <v>Tamarind Fizz</v>
-      </c>
-      <c r="B58" t="str">
-        <v>capiche</v>
-      </c>
-      <c r="C58" t="str">
-        <v>Drinks</v>
-      </c>
-      <c r="D58">
-        <v>1</v>
-      </c>
-      <c r="E58" t="str">
-        <v>Tamarind syrup</v>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="str">
-        <v>Tomato Butter Risotto</v>
-      </c>
-      <c r="B59" t="str">
-        <v>capiche</v>
-      </c>
-      <c r="C59" t="str">
-        <v>Risotto</v>
-      </c>
-      <c r="D59">
-        <v>1</v>
-      </c>
-      <c r="E59" t="str">
-        <v>Pesto dollop</v>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="str">
-        <v>Tteokbokki</v>
-      </c>
-      <c r="B60" t="str">
-        <v>aiko</v>
-      </c>
-      <c r="C60" t="str">
-        <v>Sides</v>
-      </c>
-      <c r="D60">
-        <v>1</v>
-      </c>
-      <c r="E60" t="str">
-        <v>Tteokbokki sauce</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E60"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C16"/>
   <sheetData>

</xml_diff>